<commit_message>
add geo coords loader funcition, switch between TSP and DataFrame logic
</commit_message>
<xml_diff>
--- a/math_model/data-model/Data Model.xlsx
+++ b/math_model/data-model/Data Model.xlsx
@@ -25,7 +25,7 @@
     <t>lat</t>
   </si>
   <si>
-    <t>lng</t>
+    <t>lon</t>
   </si>
   <si>
     <t>address</t>
@@ -440,7 +440,7 @@
     <xdr:ext cx="3419475" cy="2476500"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image1.png" title="Изображение"/>
+        <xdr:cNvPr id="0" name="image2.png" title="Изображение"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -468,7 +468,7 @@
     <xdr:ext cx="3419475" cy="2590800"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image2.png" title="Изображение"/>
+        <xdr:cNvPr id="0" name="image1.png" title="Изображение"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>

</xml_diff>